<commit_message>
Mise à jour automatique de la veille
</commit_message>
<xml_diff>
--- a/veille-marches-caps.xlsx
+++ b/veille-marches-caps.xlsx
@@ -413,11 +413,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
@@ -427,7 +427,7 @@
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="37" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -557,6 +557,171 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nouveau</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BOAMP test 1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Annonce test BOAMP 1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.boamp.fr</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Ajout automatique BOAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nouveau</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BOAMP test 2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Annonce test BOAMP 2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://www.boamp.fr</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Ajout automatique BOAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>nouveau</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BOAMP test 3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Annonce test BOAMP 3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.boamp.fr</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>À analyser</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Ajout automatique BOAMP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>